<commit_message>
docs: design deliverables sheet 09-Oct-2026, every screen linked
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Design Deliverables 09-Oct-2026.xlsx
+++ b/Design Deliverables 09-Oct-2026.xlsx
@@ -1961,7 +1961,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B76"/>
+  <dimension ref="A1:B84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="58" customWidth="1" min="1" max="1"/>
@@ -2047,800 +2047,896 @@
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>Consent (mobile app)</t>
+          <t>About you (mobile app)</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>https://human-optimization-lab.vercel.app/app/demo/onboarding-consent</t>
+          <t>https://human-optimization-lab.vercel.app/app/demo/onboarding-about</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Sign in after creating a password (mobile app)</t>
+          <t>Consent: records (mobile app)</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>https://human-optimization-lab.vercel.app/app/demo/onboarding-signin</t>
+          <t>https://human-optimization-lab.vercel.app/app/demo/onboarding-consent</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>Returning patient sign in (mobile app)</t>
+          <t>Consent: texts and signature (mobile app)</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>https://human-optimization-lab.vercel.app/app/demo/returning</t>
+          <t>https://human-optimization-lab.vercel.app/app/demo/onboarding-consent?to=/onboarding/consent-texts</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>Mobile App: Home (free)</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="n"/>
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Your why conversation (mobile app)</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>https://human-optimization-lab.vercel.app/app/demo/onboarding-why</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>Home</t>
+          <t>Record building (mobile app)</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>https://human-optimization-lab.vercel.app/app/demo/free</t>
+          <t>https://human-optimization-lab.vercel.app/app/demo/onboarding-syncing</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>Home: first session</t>
+          <t>Sign in after creating a password (mobile app)</t>
         </is>
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>https://human-optimization-lab.vercel.app/app/demo/free-first</t>
+          <t>https://human-optimization-lab.vercel.app/app/demo/onboarding-signin</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>Home: Dr. Patel finished the review</t>
+          <t>Returning patient sign in (mobile app)</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>https://human-optimization-lab.vercel.app/app/demo/free-checked</t>
+          <t>https://human-optimization-lab.vercel.app/app/demo/returning</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>Home: new results arrived</t>
-        </is>
-      </c>
-      <c r="B15" s="6" t="inlineStr">
-        <is>
-          <t>https://human-optimization-lab.vercel.app/app/demo/free-new-results</t>
-        </is>
-      </c>
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Mobile App: Home (free)</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>Home: readiness 3 of 5</t>
+          <t>Home</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>https://human-optimization-lab.vercel.app/app/demo/free-quiet</t>
+          <t>https://human-optimization-lab.vercel.app/app/demo/free</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>Home: readiness 2 of 5</t>
+          <t>Home: first session</t>
         </is>
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>https://human-optimization-lab.vercel.app/app/demo/free-not-ready</t>
+          <t>https://human-optimization-lab.vercel.app/app/demo/free-first</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>Home: nothing to watch</t>
+          <t>Home: Dr. Patel finished the review</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>https://human-optimization-lab.vercel.app/app/demo/free-steady</t>
+          <t>https://human-optimization-lab.vercel.app/app/demo/free-checked</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>Home: everything booked and answered</t>
+          <t>Home: new results arrived</t>
         </is>
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>https://human-optimization-lab.vercel.app/app/demo/free-caught-up</t>
+          <t>https://human-optimization-lab.vercel.app/app/demo/free-new-results</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>Home: sharing turned off</t>
+          <t>Home: readiness 3 of 5</t>
         </is>
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t>https://human-optimization-lab.vercel.app/app/demo/withdrawn</t>
+          <t>https://human-optimization-lab.vercel.app/app/demo/free-quiet</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>Home: cancelled member back on the free record</t>
+          <t>Home: readiness 2 of 5</t>
         </is>
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>https://human-optimization-lab.vercel.app/app/demo/cancelled</t>
+          <t>https://human-optimization-lab.vercel.app/app/demo/free-not-ready</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>Notifications</t>
+          <t>Home: nothing to watch</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t>https://human-optimization-lab.vercel.app/app/demo/free?to=/notifications</t>
+          <t>https://human-optimization-lab.vercel.app/app/demo/free-steady</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
-          <t>Mobile App: Record</t>
-        </is>
-      </c>
-      <c r="B23" s="4" t="n"/>
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>Home: everything booked and answered</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>https://human-optimization-lab.vercel.app/app/demo/free-caught-up</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>Record tab</t>
+          <t>Home: sharing turned off</t>
         </is>
       </c>
       <c r="B24" s="6" t="inlineStr">
         <is>
-          <t>https://human-optimization-lab.vercel.app/app/demo/free?to=/results</t>
+          <t>https://human-optimization-lab.vercel.app/app/demo/withdrawn</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>Biomarker trend (A1c)</t>
+          <t>Home: cancelled member back on the free record</t>
         </is>
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>https://human-optimization-lab.vercel.app/app/demo/free?to=/biomarker/a1c</t>
+          <t>https://human-optimization-lab.vercel.app/app/demo/cancelled</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>Biomarker trend (LDL)</t>
+          <t>Notifications</t>
         </is>
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>https://human-optimization-lab.vercel.app/app/demo/free?to=/biomarker/ldl</t>
+          <t>https://human-optimization-lab.vercel.app/app/demo/free?to=/notifications</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="5" t="inlineStr">
-        <is>
-          <t>Your medicines (with dose differences)</t>
-        </is>
-      </c>
-      <c r="B27" s="6" t="inlineStr">
-        <is>
-          <t>https://human-optimization-lab.vercel.app/app/demo/free?to=/medications</t>
-        </is>
-      </c>
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>Mobile App: Record</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>Medicine details</t>
+          <t>Record tab</t>
         </is>
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>https://human-optimization-lab.vercel.app/app/demo/free?to=/medicine/atorvastatin</t>
+          <t>https://human-optimization-lab.vercel.app/app/demo/free?to=/results</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>Visit details</t>
+          <t>Biomarker trend (A1c)</t>
         </is>
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>https://human-optimization-lab.vercel.app/app/demo/free?to=/visit/annual</t>
+          <t>https://human-optimization-lab.vercel.app/app/demo/free?to=/biomarker/a1c</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>Outside visit (urgent care)</t>
+          <t>Biomarker trend (LDL)</t>
         </is>
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>https://human-optimization-lab.vercel.app/app/demo/free?to=/visit/urgent</t>
+          <t>https://human-optimization-lab.vercel.app/app/demo/free?to=/biomarker/ldl</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>Add to your record (medicine form)</t>
+          <t>Your medicines (with dose differences)</t>
         </is>
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>https://human-optimization-lab.vercel.app/app/demo/free?to=%2Frecord%2Fadd%3Fkind%3Dmedicines</t>
+          <t>https://human-optimization-lab.vercel.app/app/demo/free?to=/medications</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>Tell us about a difference</t>
+          <t>Medicine details</t>
         </is>
       </c>
       <c r="B32" s="6" t="inlineStr">
         <is>
-          <t>https://human-optimization-lab.vercel.app/app/demo/free?to=/tell-us</t>
+          <t>https://human-optimization-lab.vercel.app/app/demo/free?to=/medicine/atorvastatin</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="3" t="inlineStr">
-        <is>
-          <t>Mobile App: To Do</t>
-        </is>
-      </c>
-      <c r="B33" s="4" t="n"/>
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Visit details</t>
+        </is>
+      </c>
+      <c r="B33" s="6" t="inlineStr">
+        <is>
+          <t>https://human-optimization-lab.vercel.app/app/demo/free?to=/visit/annual</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>To do tab</t>
+          <t>Outside visit (urgent care)</t>
         </is>
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>https://human-optimization-lab.vercel.app/app/demo/free?to=/gaps</t>
+          <t>https://human-optimization-lab.vercel.app/app/demo/free?to=/visit/urgent</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>Care gap (mammogram)</t>
+          <t>Record item details (procedure)</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>https://human-optimization-lab.vercel.app/app/demo/free?to=/task/mammogram</t>
+          <t>https://human-optimization-lab.vercel.app/app/demo/free?to=%2Frecord%2Fitem%3Fd%3D%257B%2522title%2522%253A%2522Knee%2520arthroscopy%252C%2520right%2522%252C%2522provenance%2522%253A%2522clinician%2522%252C%2522details%2522%253A%255B%255B%2522Date%2522%252C%2522Feb%25202019%2522%255D%252C%255B%2522Where%2522%252C%2522Scripps%2520Memorial%2520Hospital%2522%255D%255D%252C%2522source%2522%253A%255B%255B%2522Source%2522%252C%2522Scripps%2520Memorial%2520Hospital%2522%255D%252C%255B%2522System%2522%252C%2522Epic%2522%255D%252C%255B%2522Last%2520updated%2522%252C%2522Feb%25202019%2522%255D%255D%257D</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>Lab order</t>
+          <t>Add to your record (medicine form)</t>
         </is>
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>https://human-optimization-lab.vercel.app/app/demo/free?to=/order/labs-nov</t>
+          <t>https://human-optimization-lab.vercel.app/app/demo/free?to=%2Frecord%2Fadd%3Fkind%3Dmedicines</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
         <is>
-          <t>Book with a partner</t>
+          <t>Tell us about a difference</t>
         </is>
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>https://human-optimization-lab.vercel.app/app/demo/free?to=/book/labs-nov</t>
+          <t>https://human-optimization-lab.vercel.app/app/demo/free?to=/tell-us</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="5" t="inlineStr">
-        <is>
-          <t>Upcoming appointment</t>
-        </is>
-      </c>
-      <c r="B38" s="6" t="inlineStr">
-        <is>
-          <t>https://human-optimization-lab.vercel.app/app/demo/free?to=/visit/cardio-follow-up</t>
-        </is>
-      </c>
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>Mobile App: To Do</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
         <is>
-          <t>Record review by Dr. Patel</t>
+          <t>To do tab</t>
         </is>
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>https://human-optimization-lab.vercel.app/app/demo/free?to=/visit/review-dec</t>
+          <t>https://human-optimization-lab.vercel.app/app/demo/free?to=/gaps</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="3" t="inlineStr">
-        <is>
-          <t>Mobile App: Ask Inlay</t>
-        </is>
-      </c>
-      <c r="B40" s="4" t="n"/>
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>Care gap (mammogram)</t>
+        </is>
+      </c>
+      <c r="B40" s="6" t="inlineStr">
+        <is>
+          <t>https://human-optimization-lab.vercel.app/app/demo/free?to=/task/mammogram</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t>Ask Inlay</t>
+          <t>Lab order</t>
         </is>
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>https://human-optimization-lab.vercel.app/app/demo/free?to=/assistant</t>
+          <t>https://human-optimization-lab.vercel.app/app/demo/free?to=/order/labs-nov</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
         <is>
-          <t>AI credit nearly used</t>
+          <t>Book with a partner</t>
         </is>
       </c>
       <c r="B42" s="6" t="inlineStr">
         <is>
-          <t>https://human-optimization-lab.vercel.app/app/demo/free?to=/assistant&amp;credit=high</t>
+          <t>https://human-optimization-lab.vercel.app/app/demo/free?to=/book/labs-nov</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="5" t="inlineStr">
         <is>
-          <t>AI credit used up</t>
+          <t>Upcoming appointment</t>
         </is>
       </c>
       <c r="B43" s="6" t="inlineStr">
         <is>
-          <t>https://human-optimization-lab.vercel.app/app/demo/free?to=/assistant&amp;credit=out</t>
+          <t>https://human-optimization-lab.vercel.app/app/demo/free?to=/visit/cardio-follow-up</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="5" t="inlineStr">
         <is>
-          <t>Borrowed from next week</t>
+          <t>Record review by Dr. Patel</t>
         </is>
       </c>
       <c r="B44" s="6" t="inlineStr">
         <is>
-          <t>https://human-optimization-lab.vercel.app/app/demo/free?to=/assistant&amp;credit=borrowed</t>
+          <t>https://human-optimization-lab.vercel.app/app/demo/free?to=/visit/review-dec</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="5" t="inlineStr">
-        <is>
-          <t>Member AI credit used up</t>
-        </is>
-      </c>
-      <c r="B45" s="6" t="inlineStr">
-        <is>
-          <t>https://human-optimization-lab.vercel.app/app/demo/member?to=/assistant&amp;credit=member-out</t>
-        </is>
-      </c>
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>Mobile App: Ask Inlay</t>
+        </is>
+      </c>
+      <c r="B45" s="4" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="3" t="inlineStr">
-        <is>
-          <t>Mobile App: Upgrade and Plan Set Up</t>
-        </is>
-      </c>
-      <c r="B46" s="4" t="n"/>
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>Ask Inlay</t>
+        </is>
+      </c>
+      <c r="B46" s="6" t="inlineStr">
+        <is>
+          <t>https://human-optimization-lab.vercel.app/app/demo/free?to=/assistant</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t>Upgrade tab</t>
+          <t>AI credit nearly used</t>
         </is>
       </c>
       <c r="B47" s="6" t="inlineStr">
         <is>
-          <t>https://human-optimization-lab.vercel.app/app/demo/free?to=/plan</t>
+          <t>https://human-optimization-lab.vercel.app/app/demo/free?to=/assistant&amp;credit=high</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="5" t="inlineStr">
         <is>
-          <t>Step 1: goals</t>
+          <t>AI credit used up</t>
         </is>
       </c>
       <c r="B48" s="6" t="inlineStr">
         <is>
-          <t>https://human-optimization-lab.vercel.app/app/demo/free?to=/goals</t>
+          <t>https://human-optimization-lab.vercel.app/app/demo/free?to=/assistant&amp;credit=out</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="5" t="inlineStr">
         <is>
-          <t>Step 2: goals checked against the record</t>
+          <t>Borrowed from next week</t>
         </is>
       </c>
       <c r="B49" s="6" t="inlineStr">
         <is>
-          <t>https://human-optimization-lab.vercel.app/app/demo/free?to=/goals-record</t>
+          <t>https://human-optimization-lab.vercel.app/app/demo/free?to=/assistant&amp;credit=borrowed</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="5" t="inlineStr">
         <is>
-          <t>Step 3: health profile</t>
+          <t>Member AI credit used up</t>
         </is>
       </c>
       <c r="B50" s="6" t="inlineStr">
         <is>
-          <t>https://human-optimization-lab.vercel.app/app/demo/free?to=/health-profile</t>
+          <t>https://human-optimization-lab.vercel.app/app/demo/member?to=/assistant&amp;credit=member-out</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="5" t="inlineStr">
-        <is>
-          <t>Step 4: establish your baseline</t>
-        </is>
-      </c>
-      <c r="B51" s="6" t="inlineStr">
-        <is>
-          <t>https://human-optimization-lab.vercel.app/app/demo/free?to=/baseline</t>
-        </is>
-      </c>
+      <c r="A51" s="3" t="inlineStr">
+        <is>
+          <t>Mobile App: Upgrade and Plan Set Up</t>
+        </is>
+      </c>
+      <c r="B51" s="4" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="5" t="inlineStr">
         <is>
-          <t>Step 5: complete your enrollment</t>
+          <t>Upgrade tab</t>
         </is>
       </c>
       <c r="B52" s="6" t="inlineStr">
         <is>
-          <t>https://human-optimization-lab.vercel.app/app/demo/free?to=/enrollment</t>
+          <t>https://human-optimization-lab.vercel.app/app/demo/free?to=/plan</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="5" t="inlineStr">
         <is>
-          <t>Step 6: payment method</t>
+          <t>Step 1: goals</t>
         </is>
       </c>
       <c r="B53" s="6" t="inlineStr">
         <is>
-          <t>https://human-optimization-lab.vercel.app/app/demo/free?to=/payment</t>
+          <t>https://human-optimization-lab.vercel.app/app/demo/free?to=/goals</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="5" t="inlineStr">
         <is>
-          <t>You're enrolled</t>
+          <t>Step 2: goals checked against the record</t>
         </is>
       </c>
       <c r="B54" s="6" t="inlineStr">
         <is>
-          <t>https://human-optimization-lab.vercel.app/app/demo/member?to=/enrolled</t>
+          <t>https://human-optimization-lab.vercel.app/app/demo/free?to=/goals-record</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="5" t="inlineStr">
         <is>
-          <t>Schedule your tests</t>
+          <t>Step 3: health profile</t>
         </is>
       </c>
       <c r="B55" s="6" t="inlineStr">
         <is>
-          <t>https://human-optimization-lab.vercel.app/app/demo/member?to=/schedule-tests</t>
+          <t>https://human-optimization-lab.vercel.app/app/demo/free?to=/health-profile</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="5" t="inlineStr">
         <is>
-          <t>Your plan is ready</t>
+          <t>Step 4: establish your baseline</t>
         </is>
       </c>
       <c r="B56" s="6" t="inlineStr">
         <is>
-          <t>https://human-optimization-lab.vercel.app/app/demo/member?to=/plan-ready</t>
+          <t>https://human-optimization-lab.vercel.app/app/demo/free?to=/baseline</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="3" t="inlineStr">
-        <is>
-          <t>Mobile App: Optimization Member</t>
-        </is>
-      </c>
-      <c r="B57" s="4" t="n"/>
+      <c r="A57" s="5" t="inlineStr">
+        <is>
+          <t>Step 5: complete your enrollment</t>
+        </is>
+      </c>
+      <c r="B57" s="6" t="inlineStr">
+        <is>
+          <t>https://human-optimization-lab.vercel.app/app/demo/free?to=/enrollment</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="5" t="inlineStr">
         <is>
-          <t>Home</t>
+          <t>Step 6: payment method</t>
         </is>
       </c>
       <c r="B58" s="6" t="inlineStr">
         <is>
-          <t>https://human-optimization-lab.vercel.app/app/demo/member</t>
+          <t>https://human-optimization-lab.vercel.app/app/demo/free?to=/payment</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="5" t="inlineStr">
         <is>
-          <t>Home: bone plan</t>
+          <t>You're enrolled</t>
         </is>
       </c>
       <c r="B59" s="6" t="inlineStr">
         <is>
-          <t>https://human-optimization-lab.vercel.app/app/demo/member-bone</t>
+          <t>https://human-optimization-lab.vercel.app/app/demo/member?to=/enrolled</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="5" t="inlineStr">
         <is>
-          <t>Home: nothing logged yesterday</t>
+          <t>Schedule your tests</t>
         </is>
       </c>
       <c r="B60" s="6" t="inlineStr">
         <is>
-          <t>https://human-optimization-lab.vercel.app/app/demo/member-nothing-logged</t>
+          <t>https://human-optimization-lab.vercel.app/app/demo/member?to=/schedule-tests</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="5" t="inlineStr">
         <is>
-          <t>Home: dinner not logged</t>
+          <t>Your plan is ready</t>
         </is>
       </c>
       <c r="B61" s="6" t="inlineStr">
         <is>
-          <t>https://human-optimization-lab.vercel.app/app/demo/member-partial</t>
+          <t>https://human-optimization-lab.vercel.app/app/demo/member?to=/plan-ready</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="5" t="inlineStr">
-        <is>
-          <t>Plan version 1 with Dr. Patel</t>
-        </is>
-      </c>
-      <c r="B62" s="6" t="inlineStr">
-        <is>
-          <t>https://human-optimization-lab.vercel.app/app/demo/member-review</t>
-        </is>
-      </c>
+      <c r="A62" s="3" t="inlineStr">
+        <is>
+          <t>Mobile App: Optimization Member</t>
+        </is>
+      </c>
+      <c r="B62" s="4" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="5" t="inlineStr">
         <is>
-          <t>New plan version with Dr. Patel</t>
+          <t>Home</t>
         </is>
       </c>
       <c r="B63" s="6" t="inlineStr">
         <is>
-          <t>https://human-optimization-lab.vercel.app/app/demo/member-redraft</t>
+          <t>https://human-optimization-lab.vercel.app/app/demo/member</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="5" t="inlineStr">
         <is>
-          <t>Plan tab</t>
+          <t>Home: bone plan</t>
         </is>
       </c>
       <c r="B64" s="6" t="inlineStr">
         <is>
-          <t>https://human-optimization-lab.vercel.app/app/demo/member?to=/plan</t>
+          <t>https://human-optimization-lab.vercel.app/app/demo/member-bone</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="5" t="inlineStr">
         <is>
-          <t>Diet</t>
+          <t>Home: nothing logged yesterday</t>
         </is>
       </c>
       <c r="B65" s="6" t="inlineStr">
         <is>
-          <t>https://human-optimization-lab.vercel.app/app/demo/member?to=/diet</t>
+          <t>https://human-optimization-lab.vercel.app/app/demo/member-nothing-logged</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="5" t="inlineStr">
         <is>
-          <t>Log a meal</t>
+          <t>Home: dinner not logged</t>
         </is>
       </c>
       <c r="B66" s="6" t="inlineStr">
         <is>
-          <t>https://human-optimization-lab.vercel.app/app/demo/member?to=/log-meal</t>
+          <t>https://human-optimization-lab.vercel.app/app/demo/member-partial</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="5" t="inlineStr">
         <is>
-          <t>Exercise</t>
+          <t>Plan version 1 with Dr. Patel</t>
         </is>
       </c>
       <c r="B67" s="6" t="inlineStr">
         <is>
-          <t>https://human-optimization-lab.vercel.app/app/demo/member?to=/exercise</t>
+          <t>https://human-optimization-lab.vercel.app/app/demo/member-review</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="5" t="inlineStr">
         <is>
-          <t>Exercise move</t>
+          <t>New plan version with Dr. Patel</t>
         </is>
       </c>
       <c r="B68" s="6" t="inlineStr">
         <is>
-          <t>https://human-optimization-lab.vercel.app/app/demo/member?to=/exercise/sit-to-stand</t>
+          <t>https://human-optimization-lab.vercel.app/app/demo/member-redraft</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="5" t="inlineStr">
         <is>
-          <t>Yesterday</t>
+          <t>Plan tab</t>
         </is>
       </c>
       <c r="B69" s="6" t="inlineStr">
         <is>
-          <t>https://human-optimization-lab.vercel.app/app/demo/member?to=/day/yesterday</t>
+          <t>https://human-optimization-lab.vercel.app/app/demo/member?to=/plan</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="5" t="inlineStr">
         <is>
-          <t>Progress</t>
+          <t>Diet</t>
         </is>
       </c>
       <c r="B70" s="6" t="inlineStr">
         <is>
-          <t>https://human-optimization-lab.vercel.app/app/demo/member?to=/progress</t>
+          <t>https://human-optimization-lab.vercel.app/app/demo/member?to=/diet</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="5" t="inlineStr">
         <is>
-          <t>History</t>
+          <t>Log a meal</t>
         </is>
       </c>
       <c r="B71" s="6" t="inlineStr">
         <is>
-          <t>https://human-optimization-lab.vercel.app/app/demo/member?to=/history</t>
+          <t>https://human-optimization-lab.vercel.app/app/demo/member?to=/log-meal</t>
         </is>
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="3" t="inlineStr">
-        <is>
-          <t>Mobile App: Profile and Settings</t>
-        </is>
-      </c>
-      <c r="B72" s="4" t="n"/>
+      <c r="A72" s="5" t="inlineStr">
+        <is>
+          <t>Exercise</t>
+        </is>
+      </c>
+      <c r="B72" s="6" t="inlineStr">
+        <is>
+          <t>https://human-optimization-lab.vercel.app/app/demo/member?to=/exercise</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="5" t="inlineStr">
         <is>
-          <t>Profile</t>
+          <t>Exercise move</t>
         </is>
       </c>
       <c r="B73" s="6" t="inlineStr">
         <is>
-          <t>https://human-optimization-lab.vercel.app/app/demo/free?to=/profile</t>
+          <t>https://human-optimization-lab.vercel.app/app/demo/member?to=/exercise/sit-to-stand</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="5" t="inlineStr">
         <is>
-          <t>Access (connected records and devices)</t>
+          <t>Yesterday</t>
         </is>
       </c>
       <c r="B74" s="6" t="inlineStr">
         <is>
-          <t>https://human-optimization-lab.vercel.app/app/demo/member?to=/access</t>
+          <t>https://human-optimization-lab.vercel.app/app/demo/member?to=/day/yesterday</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="5" t="inlineStr">
         <is>
-          <t>Membership</t>
+          <t>Progress</t>
         </is>
       </c>
       <c r="B75" s="6" t="inlineStr">
         <is>
-          <t>https://human-optimization-lab.vercel.app/app/demo/member?to=/membership</t>
+          <t>https://human-optimization-lab.vercel.app/app/demo/member?to=/progress</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="5" t="inlineStr">
         <is>
+          <t>History</t>
+        </is>
+      </c>
+      <c r="B76" s="6" t="inlineStr">
+        <is>
+          <t>https://human-optimization-lab.vercel.app/app/demo/member?to=/history</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="3" t="inlineStr">
+        <is>
+          <t>Mobile App: Profile and Settings</t>
+        </is>
+      </c>
+      <c r="B77" s="4" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="5" t="inlineStr">
+        <is>
+          <t>Profile</t>
+        </is>
+      </c>
+      <c r="B78" s="6" t="inlineStr">
+        <is>
+          <t>https://human-optimization-lab.vercel.app/app/demo/free?to=/profile</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="5" t="inlineStr">
+        <is>
+          <t>Access (connected records and devices)</t>
+        </is>
+      </c>
+      <c r="B79" s="6" t="inlineStr">
+        <is>
+          <t>https://human-optimization-lab.vercel.app/app/demo/member?to=/access</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="5" t="inlineStr">
+        <is>
+          <t>Membership</t>
+        </is>
+      </c>
+      <c r="B80" s="6" t="inlineStr">
+        <is>
+          <t>https://human-optimization-lab.vercel.app/app/demo/member?to=/membership</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="5" t="inlineStr">
+        <is>
           <t>Connect your records</t>
         </is>
       </c>
-      <c r="B76" s="6" t="inlineStr">
+      <c r="B81" s="6" t="inlineStr">
         <is>
           <t>https://human-optimization-lab.vercel.app/app/demo/withdrawn?to=/connect</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="5" t="inlineStr">
+        <is>
+          <t>Connect your records: texts and signature</t>
+        </is>
+      </c>
+      <c r="B82" s="6" t="inlineStr">
+        <is>
+          <t>https://human-optimization-lab.vercel.app/app/demo/withdrawn?to=/connect-texts</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="5" t="inlineStr">
+        <is>
+          <t>Record building after connecting</t>
+        </is>
+      </c>
+      <c r="B83" s="6" t="inlineStr">
+        <is>
+          <t>https://human-optimization-lab.vercel.app/app/demo/withdrawn?to=/building</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="5" t="inlineStr">
+        <is>
+          <t>Renew sharing</t>
+        </is>
+      </c>
+      <c r="B84" s="6" t="inlineStr">
+        <is>
+          <t>https://human-optimization-lab.vercel.app/app/demo/free?to=%2Faccess%3Fsheet%3Drenew</t>
         </is>
       </c>
     </row>
@@ -2853,10 +2949,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B9" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B10" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B12" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B13" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B14" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B15" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B11" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B12" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B13" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B14" r:id="rId11"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B16" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B17" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B18" r:id="rId14"/>
@@ -2864,41 +2960,41 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B20" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B21" r:id="rId17"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B22" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B24" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B25" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B26" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B27" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B23" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B24" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B25" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B26" r:id="rId22"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B28" r:id="rId23"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B29" r:id="rId24"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B30" r:id="rId25"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B31" r:id="rId26"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B32" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B34" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B35" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B36" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B37" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B38" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B33" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B34" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B35" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B36" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B37" r:id="rId32"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B39" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B41" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B42" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B43" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B44" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B45" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B47" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B48" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B49" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B50" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B51" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B40" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B41" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B42" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B43" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B44" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B46" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B47" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B48" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B49" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B50" r:id="rId43"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B52" r:id="rId44"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B53" r:id="rId45"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B54" r:id="rId46"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B55" r:id="rId47"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B56" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B58" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B59" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B60" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B61" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B62" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B57" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B58" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B59" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B60" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B61" r:id="rId53"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B63" r:id="rId54"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B64" r:id="rId55"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B65" r:id="rId56"/>
@@ -2908,10 +3004,18 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B69" r:id="rId60"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B70" r:id="rId61"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B71" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B73" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B74" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B75" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B76" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B72" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B73" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B74" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B75" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B76" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B78" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B79" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B80" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B81" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B82" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B83" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B84" r:id="rId74"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>